<commit_message>
Rewrite Sugar News 2026-09-06 summaries
</commit_message>
<xml_diff>
--- a/reports/2026/09/Sugar News 2026-09-06.xlsx
+++ b/reports/2026/09/Sugar News 2026-09-06.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="143.35" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,16 +513,16 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度糖厂显示糖厂出厂价，糖厂出厂价为₹43、₹70。印度糖厂出厂价仅披露当前水平，缺少前期比较时不单独改变供需方向判断。来源：ChiniMandi（https://www.chinimandi.com/sugar-markets-round-trip-sugar-ex-mill-prices-erase-entire-rally-back-to-%E2%82%B943-from-%E2%82%B970-per-kg/）。影响：中性</t>
+          <t>ChiniMandi整理的印度糖厂出厂价显示，马哈拉施特拉邦西部M级糖9月5日约₹4,350/公担、北马哈拉施特拉邦约₹4,400/公担、北卡纳塔克邦约₹4,380/公担，已从此前西马哈拉施特拉邦和卡纳塔克邦接近₹70/kg的高位回落到7月中旬₹43-44/kg附近。价格回落来自印度政府9月1日起对大用户实施15天库存限制、9月15日起将经销商库存上限从4,000公担降至2,000公担，以及允许100万吨免税原糖进口，这些措施迫使超限库存释放并提高可用供应，短期利空印度现货糖价。来源：ChiniMandi（https://www.chinimandi.com/sugar-markets-round-trip-sugar-ex-mill-prices-erase-entire-rally-back-to-%E2%82%B943-from-%E2%82%B970-per-kg/）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>中性：印度糖厂出厂价仅披露当前水平，缺少前期比较时不单独改变供需方向判断。</t>
+          <t>利空：印度政府限库和100万吨免税原糖进口预期增加可流通糖源，推动糖厂出厂价从高位回落并压制短期现货糖价。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="121.9" customHeight="1" s="2">
+    <row r="3" ht="113.65" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>泰国</t>
@@ -530,16 +530,16 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>泰国气象局预报（2026-09-06），乌隆他尼、加拉信、那空沙旺、彭世洛、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
+          <t>泰国气象局9月6日预报，乌隆他尼、加拉信、那空沙旺、彭世洛、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。泰国甘蔗处于生长期，雷阵雨和局地大雨会补充土壤水分、改善甘蔗单产形成条件，提高后期甘蔗和食糖供应预期，利空糖价。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
+          <t>利空：泰国主产区生长期降雨补充土壤水分并改善甘蔗单产形成条件，提高后期甘蔗和食糖供应预期，利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="150.5" customHeight="1" s="2">
+    <row r="4" ht="180" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>巴基斯坦</t>
@@ -547,12 +547,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>巴基斯坦政府披露糖厂运行和压榨安排，披露1 million。巴基斯坦糖厂开榨、复产或压榨增加会加快当季食糖产出，增加阶段性供应。来源：Profit by Pakistan Today（https://profit.pakistantoday.com.pk/2026/09/05/farmers-body-urges-govt-to-export-1-million-tonnes-of-sugar-before-crushing-season）。影响：利空糖价</t>
+          <t>周末延续消息：巴基斯坦农民联合会（PKI）呼吁政府在11月15日新榨季开始前批准出口100万吨过剩糖，理由是国内仍有约130万吨未消费库存，且新季甘蔗产量预计增加10%-15%。巴基斯坦2025/26财年甘蔗产量已达8945万吨、同比增长6.2%，种植面积增长2.4%、平均单产780 maunds/acre；库存叠加增产预期说明国内供应压力偏大，若100万吨出口获批，将增加国际市场可供应糖源，利空国际糖价。来源：Profit by Pakistan Today（https://profit.pakistantoday.com.pk/2026/09/05/farmers-body-urges-govt-to-export-1-million-tonnes-of-sugar-before-crushing-season）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>利空：糖厂运行、压榨能力或原料供应改善会提高食糖生产节奏，增加阶段性供应。</t>
+          <t>利空：巴基斯坦现有约130万吨未消费库存且甘蔗产量预计继续增加，PKI要求出口100万吨过剩糖若获批，会把国内库存压力转化为国际市场新增供应，利空糖价。</t>
         </is>
       </c>
     </row>

</xml_diff>